<commit_message>
feat: add support for exporting `tags` field in XLSX_V3 format and update templates and tests accordingly
</commit_message>
<xml_diff>
--- a/tw-core/src/main/resources/XLSX_V3/timesheet-template.xlsx
+++ b/tw-core/src/main/resources/XLSX_V3/timesheet-template.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/tino/IdeaProjects/timesheet-wizard/tw-core/src/main/resources/XLSX_V3/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{885E4062-F6C4-C347-BA66-E3B935D33DE0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{008E6E07-1296-AF4F-92C9-720B82CF57F5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="600" windowWidth="25600" windowHeight="28200" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -62,10 +62,9 @@
         <r>
           <rPr>
             <sz val="11"/>
-            <color indexed="8"/>
+            <color rgb="FF000000"/>
             <rFont val="Aptos Narrow"/>
             <family val="2"/>
-            <scheme val="minor"/>
           </rPr>
           <t>0 oder 1</t>
         </r>
@@ -76,7 +75,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="20" uniqueCount="13">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="21" uniqueCount="13">
   <si>
     <t>Mitarbeiter</t>
   </si>
@@ -124,7 +123,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="dd\.mm\.yyyy"/>
   </numFmts>
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color indexed="8"/>
@@ -136,6 +135,12 @@
       <b/>
       <sz val="9"/>
       <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF000000"/>
+      <name val="Aptos Narrow"/>
       <family val="2"/>
     </font>
   </fonts>
@@ -576,6 +581,9 @@
       <c r="G2" t="s">
         <v>12</v>
       </c>
+      <c r="H2" t="s">
+        <v>12</v>
+      </c>
       <c r="I2" t="s">
         <v>12</v>
       </c>

</xml_diff>